<commit_message>
Common-resource items cite Krantz (2001) only; three anticipated-effects items for the ropeway
- Common-resource items: Lax & Krug removed (a working paper). Each item cites the Krantz
  (2001) passage it rests on; wording is ours. Governance has no source on disk yet.
- Module J: three parsimonious anticipated-effect items (own work, who gets the jobs, trust),
  Kedarnath route only. Concept from Pelz et al. (2024); wording ours.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kedarnath_final_kobo.xlsx
+++ b/Kedarnath_final_kobo.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O286"/>
+  <dimension ref="A1:O289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -768,7 +768,7 @@
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
         <is>
-          <t>'2026-10-05.c8aeef'</t>
+          <t>'2026-10-05.696592'</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -9475,22 +9475,22 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>select_one yn</t>
+          <t>select_one ropexp</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>trek_dependent</t>
+          <t>ropeway_expect_work</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Is your main work carrying, transporting or guiding people or goods on foot along the pilgrimage trek?</t>
+          <t>If the ropeway is built, what do you think will happen to your own work? More work for you; less work; about the same; or don't know?</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>क्या आपका मुख्य यात्रा-काम गौरीकुंड से केदारनाथ के पैदल रास्ते पर लोगों या सामान को ले जाना, पहुँचाना या रास्ता दिखाना है?</t>
+          <t>अगर रोपवे बन गया, तो आपके अपने काम पर क्या असर होगा? मेरे लिए ज़्यादा काम; मेरे लिए कम काम; लगभग वैसा ही; या पता नहीं?</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
@@ -9500,7 +9500,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H227" t="inlineStr"/>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>${site} = 1</t>
+        </is>
+      </c>
       <c r="I227" t="inlineStr"/>
       <c r="J227" t="inlineStr"/>
       <c r="K227" t="inlineStr"/>
@@ -9512,16 +9516,36 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B228" t="inlineStr"/>
-      <c r="C228" t="inlineStr"/>
-      <c r="D228" t="inlineStr"/>
+          <t>select_one ropjobs</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>ropeway_expect_jobs</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Who do you think will get most of the jobs the ropeway creates? People from these villages; people from outside the area; nobody will get jobs; or don't know?</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>रोपवे में जो नौकरियाँ बनेंगी, वे ज़्यादातर किसे मिलेंगी? इन गाँवों के लोगों को; इलाके के बाहर के लोगों को; किसी को नहीं मिलेंगी; या पता नहीं?</t>
+        </is>
+      </c>
       <c r="E228" t="inlineStr"/>
       <c r="F228" t="inlineStr"/>
-      <c r="G228" t="inlineStr"/>
-      <c r="H228" t="inlineStr"/>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>${site} = 1</t>
+        </is>
+      </c>
       <c r="I228" t="inlineStr"/>
       <c r="J228" t="inlineStr"/>
       <c r="K228" t="inlineStr"/>
@@ -9533,64 +9557,72 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>grp_K</t>
+          <t>ropeway_trust</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Module K: Job quality (Apablaza et al. 2026 questions)</t>
+          <t>Do you think the ropeway will improve the livelihoods of people here? Yes; no; or don't know?</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Module K: Job quality (Apablaza et al. 2026 questions)</t>
+          <t>क्या आपको लगता है कि रोपवे से यहाँ के लोगों की रोज़ी-रोटी सुधरेगी? हाँ; नहीं; या पता नहीं?</t>
         </is>
       </c>
       <c r="E229" t="inlineStr"/>
       <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr"/>
-      <c r="H229" t="inlineStr"/>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>${site} = 1</t>
+        </is>
+      </c>
       <c r="I229" t="inlineStr"/>
       <c r="J229" t="inlineStr"/>
       <c r="K229" t="inlineStr"/>
       <c r="L229" t="inlineStr"/>
       <c r="M229" t="inlineStr"/>
       <c r="N229" t="inlineStr"/>
-      <c r="O229" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="O229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one yn</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>intro_K</t>
+          <t>trek_dependent</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Now a set of questions about the conditions of your work — hours, pay, contract and so on. These come from a standard list used in many countries, so one or two may not fit your situation. Say so and we will move on.</t>
+          <t>Is your main work carrying, transporting or guiding people or goods on foot along the pilgrimage trek?</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>अब आपके काम के हालात पर कुछ सवाल — घंटे, मज़दूरी, ठेका वग़ैरह। ये एक बनी-बनाई सूची से हैं जो कई देशों में इस्तेमाल होती है, इसलिए एक-दो सवाल आपकी स्थिति पर शायद ठीक न बैठें। बता दीजिएगा, हम आगे बढ़ जाएँगे।</t>
+          <t>क्या आपका मुख्य यात्रा-काम गौरीकुंड से केदारनाथ के पैदल रास्ते पर लोगों या सामान को ले जाना, पहुँचाना या रास्ता दिखाना है?</t>
         </is>
       </c>
       <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr"/>
-      <c r="G230" t="inlineStr"/>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H230" t="inlineStr"/>
       <c r="I230" t="inlineStr"/>
       <c r="J230" t="inlineStr"/>
@@ -9603,39 +9635,15 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>select_one jobsit</t>
-        </is>
-      </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>job_situation</t>
-        </is>
-      </c>
-      <c r="C231" t="inlineStr">
-        <is>
-          <t>During the last month, what were you mainly doing? Ask it open and code the closest one; do not read the list out.</t>
-        </is>
-      </c>
-      <c r="D231" t="inlineStr">
-        <is>
-          <t>पिछले महीने आप मुख्य रूप से क्या कर रहे थे? खुला पूछें और जो सबसे मिलता हो वह कोड करें; पूरी सूची पढ़कर न सुनाएँ।</t>
-        </is>
-      </c>
-      <c r="E231" t="inlineStr">
-        <is>
-          <t>Code what they were MAINLY doing, by time, over the last month. Work for pay = full-time if it was their main activity on most working days, part-time or occasional if it was picked up here and there around something else. Seasonal preparation (buying stock, repairing tack, bringing animals up) IS working for pay — it is their trade — so code 1 or 2, not 10. Unemployed (8) means looking for work and not finding it; between seasons with work expected is not unemployed. Code 10 is the genuine none: not working, not studying, not looking.</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr">
-        <is>
-          <t>Code what they were MAINLY doing, by time, over the last month. Work for pay = full-time if it was their main activity on most working days, part-time or occasional if it was picked up here and there around something else. Seasonal preparation (buying stock, repairing tack, bringing animals up) IS working for pay — it is their trade — so code 1 or 2, not 10. Unemployed (8) means looking for work and not finding it; between seasons with work expected is not unemployed. Code 10 is the genuine none: not working, not studying, not looking.</t>
-        </is>
-      </c>
-      <c r="G231" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr"/>
+      <c r="C231" t="inlineStr"/>
+      <c r="D231" t="inlineStr"/>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr"/>
+      <c r="G231" t="inlineStr"/>
       <c r="H231" t="inlineStr"/>
       <c r="I231" t="inlineStr"/>
       <c r="J231" t="inlineStr"/>
@@ -9648,85 +9656,65 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>select_one jobperm</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>job_permanence</t>
+          <t>grp_K</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Is your job: permanent; seasonal or temporary; occasional or casual; on probation; or fixed-term?</t>
+          <t>Module K: Job quality (Apablaza et al. 2026 questions)</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>आपका काम कैसा है: पक्का; मौसमी या कुछ समय का; कभी-कभार का; परखने की अवधि पर; या तय समय के लिए?</t>
-        </is>
-      </c>
-      <c r="E232" t="inlineStr">
-        <is>
-          <t>Both will sound seasonal here — the Yatra closes for everyone. Ask about WITHIN the season. One employer keeps them on for a stretch = Seasonal or temporary. They take work day by day from whoever offers it = Occasional or casual. Self-employed: answer for how their own work runs. On probation and Fixed-term are rare here; do not reach for them.</t>
-        </is>
-      </c>
-      <c r="F232" t="inlineStr">
-        <is>
-          <t>यहाँ दोनों ही मौसमी लगेंगे — यात्रा तो सबके लिए बंद होती है। मौसम के अंदर की बात पूछिए। एक ही मालिक कुछ समय तक रखे हुए है = मौसमी या अस्थायी। जो भी काम रोज़-रोज़ मिल जाए वह कर लेते हैं = कभी-कभार या दिहाड़ी। अपना काम करने वालों के लिए: उनका अपना काम कैसे चलता है, वह देखिए। परख पर और तय अवधि वाले यहाँ बहुत कम मिलेंगे; इन्हें यूँ ही न चुनें।</t>
-        </is>
-      </c>
-      <c r="G232" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H232" t="inlineStr">
-        <is>
-          <t>${job_situation} &lt;= 3</t>
-        </is>
-      </c>
+          <t>Module K: Job quality (Apablaza et al. 2026 questions)</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
+      <c r="H232" t="inlineStr"/>
       <c r="I232" t="inlineStr"/>
       <c r="J232" t="inlineStr"/>
       <c r="K232" t="inlineStr"/>
       <c r="L232" t="inlineStr"/>
       <c r="M232" t="inlineStr"/>
       <c r="N232" t="inlineStr"/>
-      <c r="O232" t="inlineStr"/>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>select_one contract</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>contract_status</t>
+          <t>intro_K</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Do you have a signed contract? Yes, signed; yes but not yet signed; no contract.</t>
+          <t>Now a set of questions about the conditions of your work — hours, pay, contract and so on. These come from a standard list used in many countries, so one or two may not fit your situation. Say so and we will move on.</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>क्या आपका दस्तख़त किया हुआ अनुबंध (कॉन्ट्रैक्ट) है? हाँ, दस्तख़त किया; हाँ, पर अभी दस्तख़त नहीं हुआ; कोई अनुबंध नहीं।</t>
+          <t>अब आपके काम के हालात पर कुछ सवाल — घंटे, मज़दूरी, ठेका वग़ैरह। ये एक बनी-बनाई सूची से हैं जो कई देशों में इस्तेमाल होती है, इसलिए एक-दो सवाल आपकी स्थिति पर शायद ठीक न बैठें। बता दीजिएगा, हम आगे बढ़ जाएँगे।</t>
         </is>
       </c>
       <c r="E233" t="inlineStr"/>
       <c r="F233" t="inlineStr"/>
-      <c r="G233" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H233" t="inlineStr">
-        <is>
-          <t>(${job_situation} &lt;= 3) and (${employment_type} = 3 or ${employment_type} = 4)</t>
-        </is>
-      </c>
+      <c r="G233" t="inlineStr"/>
+      <c r="H233" t="inlineStr"/>
       <c r="I233" t="inlineStr"/>
       <c r="J233" t="inlineStr"/>
       <c r="K233" t="inlineStr"/>
@@ -9738,36 +9726,40 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>select_one yn</t>
+          <t>select_one jobsit</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>workplace_registered</t>
+          <t>job_situation</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Is your workplace or business registered, for example with a taxpayer or GST number, a shop or trade licence, the Yatra registration, or a union?</t>
+          <t>During the last month, what were you mainly doing? Ask it open and code the closest one; do not read the list out.</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>क्या आपका काम या धंधा रजिस्टर्ड है, जैसे GST या टैक्स नंबर, दुकान का लाइसेंस, यात्रा का रजिस्ट्रेशन, या कोई यूनियन?</t>
-        </is>
-      </c>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
+          <t>पिछले महीने आप मुख्य रूप से क्या कर रहे थे? खुला पूछें और जो सबसे मिलता हो वह कोड करें; पूरी सूची पढ़कर न सुनाएँ।</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Code what they were MAINLY doing, by time, over the last month. Work for pay = full-time if it was their main activity on most working days, part-time or occasional if it was picked up here and there around something else. Seasonal preparation (buying stock, repairing tack, bringing animals up) IS working for pay — it is their trade — so code 1 or 2, not 10. Unemployed (8) means looking for work and not finding it; between seasons with work expected is not unemployed. Code 10 is the genuine none: not working, not studying, not looking.</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>Code what they were MAINLY doing, by time, over the last month. Work for pay = full-time if it was their main activity on most working days, part-time or occasional if it was picked up here and there around something else. Seasonal preparation (buying stock, repairing tack, bringing animals up) IS working for pay — it is their trade — so code 1 or 2, not 10. Unemployed (8) means looking for work and not finding it; between seasons with work expected is not unemployed. Code 10 is the genuine none: not working, not studying, not looking.</t>
+        </is>
+      </c>
       <c r="G234" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="H234" t="inlineStr">
-        <is>
-          <t>${job_situation} &lt;= 3</t>
-        </is>
-      </c>
+      <c r="H234" t="inlineStr"/>
       <c r="I234" t="inlineStr"/>
       <c r="J234" t="inlineStr"/>
       <c r="K234" t="inlineStr"/>
@@ -9779,26 +9771,34 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>select_one pension</t>
+          <t>select_one jobperm</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>pension_contrib</t>
+          <t>job_permanence</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Do you contribute to any pension system? Yes, the employer deducts it; yes, voluntarily; no.</t>
+          <t>Is your job: permanent; seasonal or temporary; occasional or casual; on probation; or fixed-term?</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>क्या आप किसी पेंशन में पैसा डालते हैं? हाँ, मालिक तनख़्वाह से काटता है; हाँ, अपनी मर्ज़ी से डालते हैं; नहीं।</t>
-        </is>
-      </c>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
+          <t>आपका काम कैसा है: पक्का; मौसमी या कुछ समय का; कभी-कभार का; परखने की अवधि पर; या तय समय के लिए?</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Both will sound seasonal here — the Yatra closes for everyone. Ask about WITHIN the season. One employer keeps them on for a stretch = Seasonal or temporary. They take work day by day from whoever offers it = Occasional or casual. Self-employed: answer for how their own work runs. On probation and Fixed-term are rare here; do not reach for them.</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>यहाँ दोनों ही मौसमी लगेंगे — यात्रा तो सबके लिए बंद होती है। मौसम के अंदर की बात पूछिए। एक ही मालिक कुछ समय तक रखे हुए है = मौसमी या अस्थायी। जो भी काम रोज़-रोज़ मिल जाए वह कर लेते हैं = कभी-कभार या दिहाड़ी। अपना काम करने वालों के लिए: उनका अपना काम कैसे चलता है, वह देखिए। परख पर और तय अवधि वाले यहाँ बहुत कम मिलेंगे; इन्हें यूँ ही न चुनें।</t>
+        </is>
+      </c>
       <c r="G235" t="inlineStr">
         <is>
           <t>yes</t>
@@ -9806,7 +9806,7 @@
       </c>
       <c r="H235" t="inlineStr">
         <is>
-          <t>(${job_situation} &lt;= 3) and (${employment_type} = 3 or ${employment_type} = 4)</t>
+          <t>${job_situation} &lt;= 3</t>
         </is>
       </c>
       <c r="I235" t="inlineStr"/>
@@ -9820,22 +9820,22 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>select_one workins</t>
+          <t>select_one contract</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>work_health_ins</t>
+          <t>contract_status</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Do you have health insurance through your work? Yes; only private or other insurance; none; don't know.</t>
+          <t>Do you have a signed contract? Yes, signed; yes but not yet signed; no contract.</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>क्या काम की तरफ़ से आपका स्वास्थ्य बीमा है? हाँ; सिर्फ़ अपना या कोई और बीमा; कोई नहीं; पता नहीं।</t>
+          <t>क्या आपका दस्तख़त किया हुआ अनुबंध (कॉन्ट्रैक्ट) है? हाँ, दस्तख़त किया; हाँ, पर अभी दस्तख़त नहीं हुआ; कोई अनुबंध नहीं।</t>
         </is>
       </c>
       <c r="E236" t="inlineStr"/>
@@ -9861,22 +9861,22 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>select_one yn</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>leave_rights</t>
+          <t>workplace_registered</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Do you have the right to paid holiday, sick or maternity leave?</t>
+          <t>Is your workplace or business registered, for example with a taxpayer or GST number, a shop or trade licence, the Yatra registration, or a union?</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>क्या आपको पैसे वाली छुट्टी मिलती है — त्योहार, बीमारी या ज़च्चगी की?</t>
+          <t>क्या आपका काम या धंधा रजिस्टर्ड है, जैसे GST या टैक्स नंबर, दुकान का लाइसेंस, यात्रा का रजिस्ट्रेशन, या कोई यूनियन?</t>
         </is>
       </c>
       <c r="E237" t="inlineStr"/>
@@ -9888,7 +9888,7 @@
       </c>
       <c r="H237" t="inlineStr">
         <is>
-          <t>(${job_situation} &lt;= 3) and (${employment_type} = 3 or ${employment_type} = 4)</t>
+          <t>${job_situation} &lt;= 3</t>
         </is>
       </c>
       <c r="I237" t="inlineStr"/>
@@ -9902,22 +9902,22 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>select_one pension</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>injured_ever</t>
+          <t>pension_contrib</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Have you ever been physically injured at your workplace?</t>
+          <t>Do you contribute to any pension system? Yes, the employer deducts it; yes, voluntarily; no.</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>क्या आपको कभी काम की जगह पर चोट लगी है?</t>
+          <t>क्या आप किसी पेंशन में पैसा डालते हैं? हाँ, मालिक तनख़्वाह से काटता है; हाँ, अपनी मर्ज़ी से डालते हैं; नहीं।</t>
         </is>
       </c>
       <c r="E238" t="inlineStr"/>
@@ -9929,7 +9929,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>${job_situation} &lt;= 3</t>
+          <t>(${job_situation} &lt;= 3) and (${employment_type} = 3 or ${employment_type} = 4)</t>
         </is>
       </c>
       <c r="I238" t="inlineStr"/>
@@ -9943,22 +9943,22 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>select_one workins</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>workplace_injury_12m</t>
+          <t>work_health_ins</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>In the last 12 months, was anyone physically injured at your workplace because of work?</t>
+          <t>Do you have health insurance through your work? Yes; only private or other insurance; none; don't know.</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में क्या आपके काम की जगह पर काम की वजह से किसी को चोट लगी?</t>
+          <t>क्या काम की तरफ़ से आपका स्वास्थ्य बीमा है? हाँ; सिर्फ़ अपना या कोई और बीमा; कोई नहीं; पता नहीं।</t>
         </is>
       </c>
       <c r="E239" t="inlineStr"/>
@@ -9970,7 +9970,7 @@
       </c>
       <c r="H239" t="inlineStr">
         <is>
-          <t>${job_situation} &lt;= 3</t>
+          <t>(${job_situation} &lt;= 3) and (${employment_type} = 3 or ${employment_type} = 4)</t>
         </is>
       </c>
       <c r="I239" t="inlineStr"/>
@@ -9989,17 +9989,17 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>workplace_death_12m</t>
+          <t>leave_rights</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>And in the last 12 months, did anyone die at your workplace because of work?</t>
+          <t>Do you have the right to paid holiday, sick or maternity leave?</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>और पिछले 12 महीनों में, क्या आपके काम की जगह पर काम की वजह से किसी की मौत हुई?</t>
+          <t>क्या आपको पैसे वाली छुट्टी मिलती है — त्योहार, बीमारी या ज़च्चगी की?</t>
         </is>
       </c>
       <c r="E240" t="inlineStr"/>
@@ -10011,7 +10011,7 @@
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>${job_situation} &lt;= 3</t>
+          <t>(${job_situation} &lt;= 3) and (${employment_type} = 3 or ${employment_type} = 4)</t>
         </is>
       </c>
       <c r="I240" t="inlineStr"/>
@@ -10030,17 +10030,17 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>wants_more_work</t>
+          <t>injured_ever</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Would you like to work more hours than you do?</t>
+          <t>Have you ever been physically injured at your workplace?</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>क्या आप अभी से ज़्यादा घंटे काम करना चाहेंगे?</t>
+          <t>क्या आपको कभी काम की जगह पर चोट लगी है?</t>
         </is>
       </c>
       <c r="E241" t="inlineStr"/>
@@ -10052,7 +10052,7 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>${job_situation} &lt;= 7</t>
+          <t>${job_situation} &lt;= 3</t>
         </is>
       </c>
       <c r="I241" t="inlineStr"/>
@@ -10066,22 +10066,22 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>more_hours_day</t>
+          <t>workplace_injury_12m</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>On a working day, how many MORE hours would you like to work?</t>
+          <t>In the last 12 months, was anyone physically injured at your workplace because of work?</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
         <is>
-          <t>काम के दिन में आप कितने घंटे और काम करना चाहेंगे?</t>
+          <t>पिछले 12 महीनों में क्या आपके काम की जगह पर काम की वजह से किसी को चोट लगी?</t>
         </is>
       </c>
       <c r="E242" t="inlineStr"/>
@@ -10093,24 +10093,12 @@
       </c>
       <c r="H242" t="inlineStr">
         <is>
-          <t>${wants_more_work} = 1 or ${job_situation} = 8</t>
-        </is>
-      </c>
-      <c r="I242" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . + ${hours_day_yatra} &lt;= 18</t>
-        </is>
-      </c>
-      <c r="J242" t="inlineStr">
-        <is>
-          <t>Hours wanted plus hours already worked cannot exceed 18 in a day.</t>
-        </is>
-      </c>
-      <c r="K242" t="inlineStr">
-        <is>
-          <t>Hours wanted plus hours already worked cannot exceed 18 in a day.</t>
-        </is>
-      </c>
+          <t>${job_situation} &lt;= 3</t>
+        </is>
+      </c>
+      <c r="I242" t="inlineStr"/>
+      <c r="J242" t="inlineStr"/>
+      <c r="K242" t="inlineStr"/>
       <c r="L242" t="inlineStr"/>
       <c r="M242" t="inlineStr"/>
       <c r="N242" t="inlineStr"/>
@@ -10119,22 +10107,22 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>months_looked_for_work</t>
+          <t>workplace_death_12m</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Across the months when you had no paid work, about how many MONTHS in total were you looking for work?</t>
+          <t>And in the last 12 months, did anyone die at your workplace because of work?</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
         <is>
-          <t>जिन महीनों में आपके पास कोई पैसे वाला काम नहीं था, उनमें कुल मिलाकर लगभग कितने महीने आप काम ढूँढते रहे?</t>
+          <t>और पिछले 12 महीनों में, क्या आपके काम की जगह पर काम की वजह से किसी की मौत हुई?</t>
         </is>
       </c>
       <c r="E243" t="inlineStr"/>
@@ -10146,7 +10134,7 @@
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>${calc_months_no_work} &gt; 0 or ${job_situation} = 8</t>
+          <t>${job_situation} &lt;= 3</t>
         </is>
       </c>
       <c r="I243" t="inlineStr"/>
@@ -10165,17 +10153,17 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>first_job_ever</t>
+          <t>wants_more_work</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Was your current work the first paid job you ever had?</t>
+          <t>Would you like to work more hours than you do?</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>क्या यह आपका पहला पैसे वाला काम है?</t>
+          <t>क्या आप अभी से ज़्यादा घंटे काम करना चाहेंगे?</t>
         </is>
       </c>
       <c r="E244" t="inlineStr"/>
@@ -10185,7 +10173,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H244" t="inlineStr"/>
+      <c r="H244" t="inlineStr">
+        <is>
+          <t>${job_situation} &lt;= 7</t>
+        </is>
+      </c>
       <c r="I244" t="inlineStr"/>
       <c r="J244" t="inlineStr"/>
       <c r="K244" t="inlineStr"/>
@@ -10197,22 +10189,22 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>higher_ed</t>
+          <t>more_hours_day</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Have you completed any college, diploma or university course?</t>
+          <t>On a working day, how many MORE hours would you like to work?</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>क्या आपने कॉलेज, डिप्लोमा या यूनिवर्सिटी का कोई कोर्स पूरा किया है?</t>
+          <t>काम के दिन में आप कितने घंटे और काम करना चाहेंगे?</t>
         </is>
       </c>
       <c r="E245" t="inlineStr"/>
@@ -10224,12 +10216,24 @@
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>${job_situation} &lt;= 3</t>
-        </is>
-      </c>
-      <c r="I245" t="inlineStr"/>
-      <c r="J245" t="inlineStr"/>
-      <c r="K245" t="inlineStr"/>
+          <t>${wants_more_work} = 1 or ${job_situation} = 8</t>
+        </is>
+      </c>
+      <c r="I245" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . + ${hours_day_yatra} &lt;= 18</t>
+        </is>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Hours wanted plus hours already worked cannot exceed 18 in a day.</t>
+        </is>
+      </c>
+      <c r="K245" t="inlineStr">
+        <is>
+          <t>Hours wanted plus hours already worked cannot exceed 18 in a day.</t>
+        </is>
+      </c>
       <c r="L245" t="inlineStr"/>
       <c r="M245" t="inlineStr"/>
       <c r="N245" t="inlineStr"/>
@@ -10238,22 +10242,22 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>social_security_any</t>
+          <t>months_looked_for_work</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Are you enrolled in any pension, insurance or social-security scheme? For example, EPFO or PM-SYM pension, or Ayushman Bharat health cover.</t>
+          <t>Across the months when you had no paid work, about how many MONTHS in total were you looking for work?</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>क्या आप किसी पेंशन, बीमा या सरकारी सामाजिक सुरक्षा योजना में शामिल हैं? जैसे EPFO या PM-SYM पेंशन, या आयुष्मान भारत स्वास्थ्य कवर।</t>
+          <t>जिन महीनों में आपके पास कोई पैसे वाला काम नहीं था, उनमें कुल मिलाकर लगभग कितने महीने आप काम ढूँढते रहे?</t>
         </is>
       </c>
       <c r="E246" t="inlineStr"/>
@@ -10265,7 +10269,7 @@
       </c>
       <c r="H246" t="inlineStr">
         <is>
-          <t>${job_situation} &lt;= 3</t>
+          <t>${calc_months_no_work} &gt; 0 or ${job_situation} = 8</t>
         </is>
       </c>
       <c r="I246" t="inlineStr"/>
@@ -10284,17 +10288,17 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>intens_speed</t>
+          <t>first_job_ever</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>For more than half of your working day, do you work at very high speed?</t>
+          <t>Was your current work the first paid job you ever had?</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप बहुत तेज़ रफ़्तार से काम करते हैं?</t>
+          <t>क्या यह आपका पहला पैसे वाला काम है?</t>
         </is>
       </c>
       <c r="E247" t="inlineStr"/>
@@ -10304,11 +10308,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H247" t="inlineStr">
-        <is>
-          <t>${job_situation} &lt;= 3</t>
-        </is>
-      </c>
+      <c r="H247" t="inlineStr"/>
       <c r="I247" t="inlineStr"/>
       <c r="J247" t="inlineStr"/>
       <c r="K247" t="inlineStr"/>
@@ -10325,17 +10325,17 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>intens_deadline</t>
+          <t>higher_ed</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>For more than half of your working day, do you work to tight deadlines?</t>
+          <t>Have you completed any college, diploma or university course?</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आपको कड़ी समय-सीमा में काम करना पड़ता है?</t>
+          <t>क्या आपने कॉलेज, डिप्लोमा या यूनिवर्सिटी का कोई कोर्स पूरा किया है?</t>
         </is>
       </c>
       <c r="E248" t="inlineStr"/>
@@ -10366,17 +10366,17 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>intens_time</t>
+          <t>social_security_any</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>For more than half of your working day, do you not have enough time to finish your tasks?</t>
+          <t>Are you enrolled in any pension, insurance or social-security scheme? For example, EPFO or PM-SYM pension, or Ayushman Bharat health cover.</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आपके पास काम पूरा करने के लिए काफ़ी समय नहीं होता?</t>
+          <t>क्या आप किसी पेंशन, बीमा या सरकारी सामाजिक सुरक्षा योजना में शामिल हैं? जैसे EPFO या PM-SYM पेंशन, या आयुष्मान भारत स्वास्थ्य कवर।</t>
         </is>
       </c>
       <c r="E249" t="inlineStr"/>
@@ -10407,17 +10407,17 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>posture_position</t>
+          <t>intens_speed</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>For more than half of your working day, do you work in a tiring or painful position?</t>
+          <t>For more than half of your working day, do you work at very high speed?</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप थकाने वाली या दर्द वाली स्थिति में काम करते हैं?</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप बहुत तेज़ रफ़्तार से काम करते हैं?</t>
         </is>
       </c>
       <c r="E250" t="inlineStr"/>
@@ -10448,17 +10448,17 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>posture_loads</t>
+          <t>intens_deadline</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>For more than half of your working day, do you carry or move heavy loads?</t>
+          <t>For more than half of your working day, do you work to tight deadlines?</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप भारी बोझ उठाते या ढोते हैं?</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आपको कड़ी समय-सीमा में काम करना पड़ता है?</t>
         </is>
       </c>
       <c r="E251" t="inlineStr"/>
@@ -10489,17 +10489,17 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>posture_repetitive</t>
+          <t>intens_time</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>For more than half of your working day, do you make the same movements again and again?</t>
+          <t>For more than half of your working day, do you not have enough time to finish your tasks?</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप एक ही तरह की हरकत बार-बार करते हैं?</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आपके पास काम पूरा करने के लिए काफ़ी समय नहीं होता?</t>
         </is>
       </c>
       <c r="E252" t="inlineStr"/>
@@ -10530,17 +10530,17 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>phys_noise</t>
+          <t>posture_position</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>For more than half of your working day, are you exposed to loud noise?</t>
+          <t>For more than half of your working day, do you work in a tiring or painful position?</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप तेज़ शोर में रहते हैं?</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप थकाने वाली या दर्द वाली स्थिति में काम करते हैं?</t>
         </is>
       </c>
       <c r="E253" t="inlineStr"/>
@@ -10571,17 +10571,17 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>phys_temperature</t>
+          <t>posture_loads</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>For more than half of your working day, are you exposed to extreme heat or cold?</t>
+          <t>For more than half of your working day, do you carry or move heavy loads?</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप बहुत गर्मी या बहुत ठंड में रहते हैं?</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप भारी बोझ उठाते या ढोते हैं?</t>
         </is>
       </c>
       <c r="E254" t="inlineStr"/>
@@ -10607,16 +10607,36 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B255" t="inlineStr"/>
-      <c r="C255" t="inlineStr"/>
-      <c r="D255" t="inlineStr"/>
+          <t>select_one yndk</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>posture_repetitive</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>For more than half of your working day, do you make the same movements again and again?</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप एक ही तरह की हरकत बार-बार करते हैं?</t>
+        </is>
+      </c>
       <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr"/>
-      <c r="G255" t="inlineStr"/>
-      <c r="H255" t="inlineStr"/>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>${job_situation} &lt;= 3</t>
+        </is>
+      </c>
       <c r="I255" t="inlineStr"/>
       <c r="J255" t="inlineStr"/>
       <c r="K255" t="inlineStr"/>
@@ -10628,65 +10648,77 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>grp_L</t>
+          <t>phys_noise</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Module L: Tasks and skills (short block)</t>
+          <t>For more than half of your working day, are you exposed to loud noise?</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Module L: Tasks and skills (short block)</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप तेज़ शोर में रहते हैं?</t>
         </is>
       </c>
       <c r="E256" t="inlineStr"/>
       <c r="F256" t="inlineStr"/>
-      <c r="G256" t="inlineStr"/>
-      <c r="H256" t="inlineStr"/>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>${job_situation} &lt;= 3</t>
+        </is>
+      </c>
       <c r="I256" t="inlineStr"/>
       <c r="J256" t="inlineStr"/>
       <c r="K256" t="inlineStr"/>
       <c r="L256" t="inlineStr"/>
       <c r="M256" t="inlineStr"/>
       <c r="N256" t="inlineStr"/>
-      <c r="O256" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="O256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>intro_L</t>
+          <t>phys_temperature</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Last, I will read out some kinds of work-tasks and ask whether you do them. There is no right or wrong answer — we are trying to understand what skills the work here actually uses.</t>
+          <t>For more than half of your working day, are you exposed to extreme heat or cold?</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>आख़िर में, मैं कुछ तरह के कामों के नाम पढ़ूँगा और पूछूँगा कि आप वे करते हैं या नहीं। इसमें सही या ग़लत जवाब कुछ नहीं है — हम बस यह समझना चाहते हैं कि यहाँ के काम में कौन-कौन से हुनर लगते हैं।</t>
+          <t>काम के दिन के आधे से ज़्यादा समय, क्या आप बहुत गर्मी या बहुत ठंड में रहते हैं?</t>
         </is>
       </c>
       <c r="E257" t="inlineStr"/>
       <c r="F257" t="inlineStr"/>
-      <c r="G257" t="inlineStr"/>
-      <c r="H257" t="inlineStr"/>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>${job_situation} &lt;= 3</t>
+        </is>
+      </c>
       <c r="I257" t="inlineStr"/>
       <c r="J257" t="inlineStr"/>
       <c r="K257" t="inlineStr"/>
@@ -10698,31 +10730,15 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>select_one task3</t>
-        </is>
-      </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>tk_load</t>
-        </is>
-      </c>
-      <c r="C258" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Do you load, unload, stack or count goods? </t>
-        </is>
-      </c>
-      <c r="D258" t="inlineStr">
-        <is>
-          <t>क्या आप सामान चढ़ाना-उतारना, लगाना या गिनना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr"/>
+      <c r="C258" t="inlineStr"/>
+      <c r="D258" t="inlineStr"/>
       <c r="E258" t="inlineStr"/>
       <c r="F258" t="inlineStr"/>
-      <c r="G258" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G258" t="inlineStr"/>
       <c r="H258" t="inlineStr"/>
       <c r="I258" t="inlineStr"/>
       <c r="J258" t="inlineStr"/>
@@ -10735,31 +10751,27 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>select_one task3</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>tk_drive</t>
+          <t>grp_L</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you drive a motor vehicle? </t>
+          <t>Module L: Tasks and skills (short block)</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>क्या आप गाड़ी चलाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>Module L: Tasks and skills (short block)</t>
         </is>
       </c>
       <c r="E259" t="inlineStr"/>
       <c r="F259" t="inlineStr"/>
-      <c r="G259" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G259" t="inlineStr"/>
       <c r="H259" t="inlineStr"/>
       <c r="I259" t="inlineStr"/>
       <c r="J259" t="inlineStr"/>
@@ -10767,36 +10779,36 @@
       <c r="L259" t="inlineStr"/>
       <c r="M259" t="inlineStr"/>
       <c r="N259" t="inlineStr"/>
-      <c r="O259" t="inlineStr"/>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>select_one task3</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>tk_engine</t>
+          <t>intro_L</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you operate an engine or machine? </t>
+          <t>Last, I will read out some kinds of work-tasks and ask whether you do them. There is no right or wrong answer — we are trying to understand what skills the work here actually uses.</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>क्या आप इंजन या मशीन चलाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>आख़िर में, मैं कुछ तरह के कामों के नाम पढ़ूँगा और पूछूँगा कि आप वे करते हैं या नहीं। इसमें सही या ग़लत जवाब कुछ नहीं है — हम बस यह समझना चाहते हैं कि यहाँ के काम में कौन-कौन से हुनर लगते हैं।</t>
         </is>
       </c>
       <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr"/>
-      <c r="G260" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G260" t="inlineStr"/>
       <c r="H260" t="inlineStr"/>
       <c r="I260" t="inlineStr"/>
       <c r="J260" t="inlineStr"/>
@@ -10814,17 +10826,17 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>tk_electric</t>
+          <t>tk_load</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you do electrical or wiring work? </t>
+          <t xml:space="preserve">Do you load, unload, stack or count goods? </t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>क्या आप बिजली या तार का काम करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप सामान चढ़ाना-उतारना, लगाना या गिनना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E261" t="inlineStr"/>
@@ -10851,17 +10863,17 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>tk_safety</t>
+          <t>tk_drive</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you check equipment or the route for safety? </t>
+          <t xml:space="preserve">Do you drive a motor vehicle? </t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>क्या आप सामान या रास्ते की सुरक्षा जाँचना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप गाड़ी चलाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E262" t="inlineStr"/>
@@ -10888,17 +10900,17 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>tk_sell</t>
+          <t>tk_engine</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you sell goods or services? </t>
+          <t xml:space="preserve">Do you operate an engine or machine? </t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>क्या आप सामान या सेवा बेचना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप इंजन या मशीन चलाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E263" t="inlineStr"/>
@@ -10925,17 +10937,17 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>tk_cash</t>
+          <t>tk_electric</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you handle cash and payments? </t>
+          <t xml:space="preserve">Do you do electrical or wiring work? </t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>क्या आप पैसे और भुगतान सँभालना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप बिजली या तार का काम करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E264" t="inlineStr"/>
@@ -10962,17 +10974,17 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>tk_cook</t>
+          <t>tk_safety</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you cook or prepare food or drink? </t>
+          <t xml:space="preserve">Do you check equipment or the route for safety? </t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>क्या आप खाना या पीने की चीज़ बनाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप सामान या रास्ते की सुरक्षा जाँचना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E265" t="inlineStr"/>
@@ -10999,17 +11011,17 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>tk_serve</t>
+          <t>tk_sell</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you serve guests or customers? </t>
+          <t xml:space="preserve">Do you sell goods or services? </t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>क्या आप मेहमानों या ग्राहकों की सेवा करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप सामान या सेवा बेचना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E266" t="inlineStr"/>
@@ -11036,17 +11048,17 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>tk_clean</t>
+          <t>tk_cash</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you clean rooms or public areas? </t>
+          <t xml:space="preserve">Do you handle cash and payments? </t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>क्या आप कमरे या सार्वजनिक जगह साफ़ करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप पैसे और भुगतान सँभालना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E267" t="inlineStr"/>
@@ -11073,17 +11085,17 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>tk_guide</t>
+          <t>tk_cook</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you guide or explain things to visitors? </t>
+          <t xml:space="preserve">Do you cook or prepare food or drink? </t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>क्या आप आने वालों को रास्ता या बात समझाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप खाना या पीने की चीज़ बनाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E268" t="inlineStr"/>
@@ -11110,17 +11122,17 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>tk_coord</t>
+          <t>tk_serve</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Do you coordinate work by phone, radio or signals? </t>
+          <t xml:space="preserve">Do you serve guests or customers? </t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>क्या आप फ़ोन, रेडियो या इशारों से दूसरों के साथ तालमेल करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
+          <t>क्या आप मेहमानों या ग्राहकों की सेवा करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E269" t="inlineStr"/>
@@ -11142,22 +11154,22 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>select_one yn</t>
+          <t>select_one task3</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>drove_twowheeler</t>
+          <t>tk_clean</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Have you ever driven a motorcycle or scooter, with or without a licence?</t>
+          <t xml:space="preserve">Do you clean rooms or public areas? </t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>क्या आपने कभी मोटरसाइकिल या स्कूटर चलाई है, लाइसेंस हो या न हो?</t>
+          <t>क्या आप कमरे या सार्वजनिक जगह साफ़ करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E270" t="inlineStr"/>
@@ -11167,11 +11179,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr">
-        <is>
-          <t>${tk_drive} = 1 or ${tk_drive} = 2</t>
-        </is>
-      </c>
+      <c r="H270" t="inlineStr"/>
       <c r="I270" t="inlineStr"/>
       <c r="J270" t="inlineStr"/>
       <c r="K270" t="inlineStr"/>
@@ -11183,22 +11191,22 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>select_one yn</t>
+          <t>select_one task3</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>drove_car</t>
+          <t>tk_guide</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>... a car or jeep?</t>
+          <t xml:space="preserve">Do you guide or explain things to visitors? </t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>...कार या जीप?</t>
+          <t>क्या आप आने वालों को रास्ता या बात समझाना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E271" t="inlineStr"/>
@@ -11208,11 +11216,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr">
-        <is>
-          <t>${tk_drive} = 1 or ${tk_drive} = 2</t>
-        </is>
-      </c>
+      <c r="H271" t="inlineStr"/>
       <c r="I271" t="inlineStr"/>
       <c r="J271" t="inlineStr"/>
       <c r="K271" t="inlineStr"/>
@@ -11224,22 +11228,22 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>select_one yn</t>
+          <t>select_one task3</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>drove_heavy</t>
+          <t>tk_coord</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>... a truck or bus?</t>
+          <t xml:space="preserve">Do you coordinate work by phone, radio or signals? </t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>...ट्रक या बस?</t>
+          <t>क्या आप फ़ोन, रेडियो या इशारों से दूसरों के साथ तालमेल करना का काम करते हैं? (1 अपने मुख्य यात्रा-काम में नियमित; 2 मुख्य काम में नहीं, पर पहले कहीं और किया है; 3 कभी नहीं)</t>
         </is>
       </c>
       <c r="E272" t="inlineStr"/>
@@ -11249,11 +11253,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr">
-        <is>
-          <t>${tk_drive} = 1 or ${tk_drive} = 2</t>
-        </is>
-      </c>
+      <c r="H272" t="inlineStr"/>
       <c r="I272" t="inlineStr"/>
       <c r="J272" t="inlineStr"/>
       <c r="K272" t="inlineStr"/>
@@ -11270,17 +11270,17 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>read_at_work</t>
+          <t>drove_twowheeler</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>In your work, do you read anything (notes, rate lists, tickets, messages)?</t>
+          <t>Have you ever driven a motorcycle or scooter, with or without a licence?</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>अपने काम में क्या आप कुछ पढ़ते हैं (पर्ची, रेट लिस्ट, टिकट, मैसेज)?</t>
+          <t>क्या आपने कभी मोटरसाइकिल या स्कूटर चलाई है, लाइसेंस हो या न हो?</t>
         </is>
       </c>
       <c r="E273" t="inlineStr"/>
@@ -11290,7 +11290,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr"/>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>${tk_drive} = 1 or ${tk_drive} = 2</t>
+        </is>
+      </c>
       <c r="I273" t="inlineStr"/>
       <c r="J273" t="inlineStr"/>
       <c r="K273" t="inlineStr"/>
@@ -11307,17 +11311,17 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>calc_at_work</t>
+          <t>drove_car</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>In your work, do you work out prices or costs?</t>
+          <t>... a car or jeep?</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>अपने काम में क्या आप दाम या ख़र्चा जोड़ते-घटाते हैं?</t>
+          <t>...कार या जीप?</t>
         </is>
       </c>
       <c r="E274" t="inlineStr"/>
@@ -11327,7 +11331,11 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr"/>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>${tk_drive} = 1 or ${tk_drive} = 2</t>
+        </is>
+      </c>
       <c r="I274" t="inlineStr"/>
       <c r="J274" t="inlineStr"/>
       <c r="K274" t="inlineStr"/>
@@ -11339,16 +11347,36 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr"/>
-      <c r="C275" t="inlineStr"/>
-      <c r="D275" t="inlineStr"/>
+          <t>select_one yn</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>drove_heavy</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>... a truck or bus?</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>...ट्रक या बस?</t>
+        </is>
+      </c>
       <c r="E275" t="inlineStr"/>
       <c r="F275" t="inlineStr"/>
-      <c r="G275" t="inlineStr"/>
-      <c r="H275" t="inlineStr"/>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>${tk_drive} = 1 or ${tk_drive} = 2</t>
+        </is>
+      </c>
       <c r="I275" t="inlineStr"/>
       <c r="J275" t="inlineStr"/>
       <c r="K275" t="inlineStr"/>
@@ -11360,27 +11388,31 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one yn</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>grp_M</t>
+          <t>read_at_work</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Module M: Access to common resources (short block)</t>
+          <t>In your work, do you read anything (notes, rate lists, tickets, messages)?</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>Module M: Access to common resources (short block)</t>
+          <t>अपने काम में क्या आप कुछ पढ़ते हैं (पर्ची, रेट लिस्ट, टिकट, मैसेज)?</t>
         </is>
       </c>
       <c r="E276" t="inlineStr"/>
       <c r="F276" t="inlineStr"/>
-      <c r="G276" t="inlineStr"/>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H276" t="inlineStr"/>
       <c r="I276" t="inlineStr"/>
       <c r="J276" t="inlineStr"/>
@@ -11388,31 +11420,27 @@
       <c r="L276" t="inlineStr"/>
       <c r="M276" t="inlineStr"/>
       <c r="N276" t="inlineStr"/>
-      <c r="O276" t="inlineStr">
-        <is>
-          <t>field-list</t>
-        </is>
-      </c>
+      <c r="O276" t="inlineStr"/>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>select_one yn</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>cpr_firewood</t>
+          <t>calc_at_work</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>In the last 12 months, did anyone in your household collect firewood or dead wood from common land or forest near here?</t>
+          <t>In your work, do you work out prices or costs?</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने आस-पास की साझा ज़मीन या जंगल से लकड़ी या सूखी टहनियाँ इकट्ठी कीं?</t>
+          <t>अपने काम में क्या आप दाम या ख़र्चा जोड़ते-घटाते हैं?</t>
         </is>
       </c>
       <c r="E277" t="inlineStr"/>
@@ -11434,31 +11462,15 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>cpr_fodder</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t>In the last 12 months, did anyone in your household cut grass or fodder from common land near here?</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने साझा ज़मीन से घास या चारा काटा?</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr"/>
+      <c r="C278" t="inlineStr"/>
+      <c r="D278" t="inlineStr"/>
       <c r="E278" t="inlineStr"/>
       <c r="F278" t="inlineStr"/>
-      <c r="G278" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G278" t="inlineStr"/>
       <c r="H278" t="inlineStr"/>
       <c r="I278" t="inlineStr"/>
       <c r="J278" t="inlineStr"/>
@@ -11471,31 +11483,27 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>select_one yndk</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>cpr_forest_produce</t>
+          <t>grp_M</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>In the last 12 months, did anyone in your household collect herbs, mushrooms or wild fruit from the forest?</t>
+          <t>Module M: Access to common resources (short block)</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने जंगल से जड़ी-बूटी, मशरूम या जंगली फल इकट्ठे किए?</t>
+          <t>Module M: Access to common resources (short block)</t>
         </is>
       </c>
       <c r="E279" t="inlineStr"/>
       <c r="F279" t="inlineStr"/>
-      <c r="G279" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
+      <c r="G279" t="inlineStr"/>
       <c r="H279" t="inlineStr"/>
       <c r="I279" t="inlineStr"/>
       <c r="J279" t="inlineStr"/>
@@ -11503,7 +11511,11 @@
       <c r="L279" t="inlineStr"/>
       <c r="M279" t="inlineStr"/>
       <c r="N279" t="inlineStr"/>
-      <c r="O279" t="inlineStr"/>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>field-list</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -11513,17 +11525,17 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>cpr_grazing</t>
+          <t>cpr_firewood</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>In the last 12 months, did any animal of your household graze on common pasture?</t>
+          <t>In the last 12 months, did anyone in your household collect firewood or dead wood from common land or forest near here?</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर का कोई जानवर साझा चरागाह में चरा?</t>
+          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने आस-पास की साझा ज़मीन या जंगल से लकड़ी या सूखी टहनियाँ इकट्ठी कीं?</t>
         </is>
       </c>
       <c r="E280" t="inlineStr"/>
@@ -11550,17 +11562,17 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>cpr_restricted</t>
+          <t>cpr_fodder</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>In the last 12 months, has anyone in your household been stopped from using a common forest, pasture or path, or been asked to pay to use it?</t>
+          <t>In the last 12 months, did anyone in your household cut grass or fodder from common land near here?</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी को साझा जंगल, चरागाह या रास्ते के इस्तेमाल से रोका गया, या इसके लिए पैसे देने को कहा गया?</t>
+          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने साझा ज़मीन से घास या चारा काटा?</t>
         </is>
       </c>
       <c r="E281" t="inlineStr"/>
@@ -11587,17 +11599,17 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>cpr_lost_access</t>
+          <t>cpr_forest_produce</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>In the last 12 months, has a common place you used to collect from or graze on been closed because of building, road or ropeway work?</t>
+          <t>In the last 12 months, did anyone in your household collect herbs, mushrooms or wild fruit from the forest?</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या कोई साझा जगह, जहाँ आप पहले लकड़ी, घास या चारा लेते थे, निर्माण, सड़क या रोपवे के काम की वजह से बंद हो गई?</t>
+          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने जंगल से जड़ी-बूटी, मशरूम या जंगली फल इकट्ठे किए?</t>
         </is>
       </c>
       <c r="E282" t="inlineStr"/>
@@ -11619,22 +11631,22 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>select_one cprwater</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>cpr_water_route</t>
+          <t>cpr_grazing</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>On your route or near your worksite, can you use a common water source (spring, tap or stream) without paying?</t>
+          <t>In the last 12 months, did any animal of your household graze on common pasture?</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>रास्ते पर या काम की जगह के पास, क्या आप कोई साझा पानी का स्रोत (झरना, नल या नदी-नाला) बिना पैसे दिए इस्तेमाल कर सकते हैं?</t>
+          <t>पिछले 12 महीनों में, क्या आपके घर का कोई जानवर साझा चरागाह में चरा?</t>
         </is>
       </c>
       <c r="E283" t="inlineStr"/>
@@ -11656,22 +11668,22 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>select_one cprgov</t>
+          <t>select_one yndk</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>cpr_governance</t>
+          <t>cpr_restricted</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>In this area, who decides who may use the common land and forest? Ask and code what they name; do not read the list.</t>
+          <t>In the last 12 months, has anyone in your household been stopped from using a common forest, pasture or path, or been asked to pay to use it?</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>इस इलाके की साझा ज़मीन और जंगल का फ़ैसला कौन करता है, कि कौन उसका इस्तेमाल कर सकता है? जो नाम लें वही लिख लें; सूची न पढ़ें।</t>
+          <t>पिछले 12 महीनों में, क्या आपके घर के किसी को साझा जंगल, चरागाह या रास्ते के इस्तेमाल से रोका गया, या इसके लिए पैसे देने को कहा गया?</t>
         </is>
       </c>
       <c r="E284" t="inlineStr"/>
@@ -11693,15 +11705,31 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B285" t="inlineStr"/>
-      <c r="C285" t="inlineStr"/>
-      <c r="D285" t="inlineStr"/>
+          <t>select_one yndk</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>cpr_lost_access</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>In the last 12 months, has a common place you used to collect from or graze on been closed because of building, road or ropeway work?</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>पिछले 12 महीनों में, क्या कोई साझा जगह, जहाँ आप पहले लकड़ी, घास या चारा लेते थे, निर्माण, सड़क या रोपवे के काम की वजह से बंद हो गई?</t>
+        </is>
+      </c>
       <c r="E285" t="inlineStr"/>
       <c r="F285" t="inlineStr"/>
-      <c r="G285" t="inlineStr"/>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H285" t="inlineStr"/>
       <c r="I285" t="inlineStr"/>
       <c r="J285" t="inlineStr"/>
@@ -11714,15 +11742,31 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B286" t="inlineStr"/>
-      <c r="C286" t="inlineStr"/>
-      <c r="D286" t="inlineStr"/>
+          <t>select_one cprwater</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>cpr_water_route</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>On your route or near your worksite, can you use a common water source (spring, tap or stream) without paying?</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>रास्ते पर या काम की जगह के पास, क्या आप कोई साझा पानी का स्रोत (झरना, नल या नदी-नाला) बिना पैसे दिए इस्तेमाल कर सकते हैं?</t>
+        </is>
+      </c>
       <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr"/>
-      <c r="G286" t="inlineStr"/>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H286" t="inlineStr"/>
       <c r="I286" t="inlineStr"/>
       <c r="J286" t="inlineStr"/>
@@ -11731,6 +11775,85 @@
       <c r="M286" t="inlineStr"/>
       <c r="N286" t="inlineStr"/>
       <c r="O286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>select_one cprgov</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>cpr_governance</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>In this area, who decides who may use the common land and forest? Ask and code what they name; do not read the list.</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>इस इलाके की साझा ज़मीन और जंगल का फ़ैसला कौन करता है, कि कौन उसका इस्तेमाल कर सकता है? जो नाम लें वही लिख लें; सूची न पढ़ें।</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr"/>
+      <c r="I287" t="inlineStr"/>
+      <c r="J287" t="inlineStr"/>
+      <c r="K287" t="inlineStr"/>
+      <c r="L287" t="inlineStr"/>
+      <c r="M287" t="inlineStr"/>
+      <c r="N287" t="inlineStr"/>
+      <c r="O287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr"/>
+      <c r="C288" t="inlineStr"/>
+      <c r="D288" t="inlineStr"/>
+      <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="inlineStr"/>
+      <c r="H288" t="inlineStr"/>
+      <c r="I288" t="inlineStr"/>
+      <c r="J288" t="inlineStr"/>
+      <c r="K288" t="inlineStr"/>
+      <c r="L288" t="inlineStr"/>
+      <c r="M288" t="inlineStr"/>
+      <c r="N288" t="inlineStr"/>
+      <c r="O288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr"/>
+      <c r="C289" t="inlineStr"/>
+      <c r="D289" t="inlineStr"/>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="inlineStr"/>
+      <c r="H289" t="inlineStr"/>
+      <c r="I289" t="inlineStr"/>
+      <c r="J289" t="inlineStr"/>
+      <c r="K289" t="inlineStr"/>
+      <c r="L289" t="inlineStr"/>
+      <c r="M289" t="inlineStr"/>
+      <c r="N289" t="inlineStr"/>
+      <c r="O289" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11743,7 +11866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E327"/>
+  <dimension ref="A1:E335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17503,7 +17626,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>ruralurban</t>
+          <t>ropexp</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -17511,12 +17634,12 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Village (rural)</t>
+          <t>More work for me</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>गाँव में</t>
+          <t>मेरे लिए ज़्यादा काम</t>
         </is>
       </c>
       <c r="E251" t="n">
@@ -17526,7 +17649,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>ruralurban</t>
+          <t>ropexp</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -17534,12 +17657,12 @@
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Town or city (urban)</t>
+          <t>Less work for me</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>शहर या क़स्बे में</t>
+          <t>मेरे लिए कम काम</t>
         </is>
       </c>
       <c r="E252" t="n">
@@ -17549,53 +17672,53 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>ropexp</t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Male</t>
+          <t>About the same</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>पुरुष</t>
+          <t>लगभग वैसा ही</t>
         </is>
       </c>
       <c r="E253" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>sex</t>
+          <t>ropexp</t>
         </is>
       </c>
       <c r="B254" t="n">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Female</t>
+          <t>Don't know</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>महिला</t>
+          <t>पता नहीं</t>
         </is>
       </c>
       <c r="E254" t="n">
-        <v>1</v>
+        <v>97</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>ropjobs</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -17603,12 +17726,12 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Kedarnath (Gaurikund to Kedarnath)</t>
+          <t>People from these villages</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>केदारनाथ (गौरीकुंड से केदारनाथ)</t>
+          <t>इन गाँवों के लोगों को</t>
         </is>
       </c>
       <c r="E255" t="n">
@@ -17618,7 +17741,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>site</t>
+          <t>ropjobs</t>
         </is>
       </c>
       <c r="B256" t="n">
@@ -17626,12 +17749,12 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Hemkund Sahib (Govindghat to Hemkund)</t>
+          <t>People from outside the area</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>हेमकुंड साहिब (गोविंदघाट से हेमकुंड)</t>
+          <t>इलाके के बाहर के लोगों को</t>
         </is>
       </c>
       <c r="E256" t="n">
@@ -17641,277 +17764,277 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>ropjobs</t>
         </is>
       </c>
       <c r="B257" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Support</t>
+          <t>Nobody will get jobs</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>समर्थन में</t>
+          <t>किसी को नहीं मिलेंगी</t>
         </is>
       </c>
       <c r="E257" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>ropjobs</t>
         </is>
       </c>
       <c r="B258" t="n">
-        <v>2</v>
+        <v>97</v>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Don't know</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>तटस्थ</t>
+          <t>पता नहीं</t>
         </is>
       </c>
       <c r="E258" t="n">
-        <v>2</v>
+        <v>97</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>ruralurban</t>
         </is>
       </c>
       <c r="B259" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Oppose</t>
+          <t>Village (rural)</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>विरोध में</t>
+          <t>गाँव में</t>
         </is>
       </c>
       <c r="E259" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>stance</t>
+          <t>ruralurban</t>
         </is>
       </c>
       <c r="B260" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Prefer not to say</t>
+          <t>Town or city (urban)</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>बताना नहीं चाहते</t>
+          <t>शहर या क़स्बे में</t>
         </is>
       </c>
       <c r="E260" t="n">
-        <v>98</v>
+        <v>2</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="B261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Andhra Pradesh</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>आंध्र प्रदेश</t>
+          <t>पुरुष</t>
         </is>
       </c>
       <c r="E261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>sex</t>
         </is>
       </c>
       <c r="B262" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Arunachal Pradesh</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>अरुणाचल प्रदेश</t>
+          <t>महिला</t>
         </is>
       </c>
       <c r="E262" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>site</t>
         </is>
       </c>
       <c r="B263" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Assam</t>
+          <t>Kedarnath (Gaurikund to Kedarnath)</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>असम</t>
+          <t>केदारनाथ (गौरीकुंड से केदारनाथ)</t>
         </is>
       </c>
       <c r="E263" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>site</t>
         </is>
       </c>
       <c r="B264" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Bihar</t>
+          <t>Hemkund Sahib (Govindghat to Hemkund)</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>बिहार</t>
+          <t>हेमकुंड साहिब (गोविंदघाट से हेमकुंड)</t>
         </is>
       </c>
       <c r="E264" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>stance</t>
         </is>
       </c>
       <c r="B265" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Chhattisgarh</t>
+          <t>Support</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>छत्तीसगढ़</t>
+          <t>समर्थन में</t>
         </is>
       </c>
       <c r="E265" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>stance</t>
         </is>
       </c>
       <c r="B266" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Goa</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>गोवा</t>
+          <t>तटस्थ</t>
         </is>
       </c>
       <c r="E266" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>stance</t>
         </is>
       </c>
       <c r="B267" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Gujarat</t>
+          <t>Oppose</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>गुजरात</t>
+          <t>विरोध में</t>
         </is>
       </c>
       <c r="E267" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>state</t>
+          <t>stance</t>
         </is>
       </c>
       <c r="B268" t="n">
-        <v>8</v>
+        <v>98</v>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Haryana</t>
+          <t>Prefer not to say</t>
         </is>
       </c>
       <c r="D268" t="inlineStr">
         <is>
-          <t>हरियाणा</t>
+          <t>बताना नहीं चाहते</t>
         </is>
       </c>
       <c r="E268" t="n">
-        <v>8</v>
+        <v>98</v>
       </c>
     </row>
     <row r="269">
@@ -17921,20 +18044,20 @@
         </is>
       </c>
       <c r="B269" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Himachal Pradesh</t>
+          <t>Andhra Pradesh</t>
         </is>
       </c>
       <c r="D269" t="inlineStr">
         <is>
-          <t>हिमाचल प्रदेश</t>
+          <t>आंध्र प्रदेश</t>
         </is>
       </c>
       <c r="E269" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="270">
@@ -17944,20 +18067,20 @@
         </is>
       </c>
       <c r="B270" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Jharkhand</t>
+          <t>Arunachal Pradesh</t>
         </is>
       </c>
       <c r="D270" t="inlineStr">
         <is>
-          <t>झारखंड</t>
+          <t>अरुणाचल प्रदेश</t>
         </is>
       </c>
       <c r="E270" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
     </row>
     <row r="271">
@@ -17967,20 +18090,20 @@
         </is>
       </c>
       <c r="B271" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Assam</t>
         </is>
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>कर्नाटक</t>
+          <t>असम</t>
         </is>
       </c>
       <c r="E271" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="272">
@@ -17990,20 +18113,20 @@
         </is>
       </c>
       <c r="B272" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Bihar</t>
         </is>
       </c>
       <c r="D272" t="inlineStr">
         <is>
-          <t>केरल</t>
+          <t>बिहार</t>
         </is>
       </c>
       <c r="E272" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="273">
@@ -18013,20 +18136,20 @@
         </is>
       </c>
       <c r="B273" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Madhya Pradesh</t>
+          <t>Chhattisgarh</t>
         </is>
       </c>
       <c r="D273" t="inlineStr">
         <is>
-          <t>मध्य प्रदेश</t>
+          <t>छत्तीसगढ़</t>
         </is>
       </c>
       <c r="E273" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="274">
@@ -18036,20 +18159,20 @@
         </is>
       </c>
       <c r="B274" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Maharashtra</t>
+          <t>Goa</t>
         </is>
       </c>
       <c r="D274" t="inlineStr">
         <is>
-          <t>महाराष्ट्र</t>
+          <t>गोवा</t>
         </is>
       </c>
       <c r="E274" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
     </row>
     <row r="275">
@@ -18059,20 +18182,20 @@
         </is>
       </c>
       <c r="B275" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Manipur</t>
+          <t>Gujarat</t>
         </is>
       </c>
       <c r="D275" t="inlineStr">
         <is>
-          <t>मणिपुर</t>
+          <t>गुजरात</t>
         </is>
       </c>
       <c r="E275" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
     </row>
     <row r="276">
@@ -18082,20 +18205,20 @@
         </is>
       </c>
       <c r="B276" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Meghalaya</t>
+          <t>Haryana</t>
         </is>
       </c>
       <c r="D276" t="inlineStr">
         <is>
-          <t>मेघालय</t>
+          <t>हरियाणा</t>
         </is>
       </c>
       <c r="E276" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="277">
@@ -18105,20 +18228,20 @@
         </is>
       </c>
       <c r="B277" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Mizoram</t>
+          <t>Himachal Pradesh</t>
         </is>
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>मिज़ोरम</t>
+          <t>हिमाचल प्रदेश</t>
         </is>
       </c>
       <c r="E277" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="278">
@@ -18128,20 +18251,20 @@
         </is>
       </c>
       <c r="B278" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Nagaland</t>
+          <t>Jharkhand</t>
         </is>
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>नागालैंड</t>
+          <t>झारखंड</t>
         </is>
       </c>
       <c r="E278" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="279">
@@ -18151,20 +18274,20 @@
         </is>
       </c>
       <c r="B279" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Odisha</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>ओडिशा</t>
+          <t>कर्नाटक</t>
         </is>
       </c>
       <c r="E279" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="280">
@@ -18174,20 +18297,20 @@
         </is>
       </c>
       <c r="B280" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Punjab</t>
+          <t>Kerala</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>पंजाब</t>
+          <t>केरल</t>
         </is>
       </c>
       <c r="E280" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="281">
@@ -18197,20 +18320,20 @@
         </is>
       </c>
       <c r="B281" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>Rajasthan</t>
+          <t>Madhya Pradesh</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>राजस्थान</t>
+          <t>मध्य प्रदेश</t>
         </is>
       </c>
       <c r="E281" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="282">
@@ -18220,20 +18343,20 @@
         </is>
       </c>
       <c r="B282" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Sikkim</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>सिक्किम</t>
+          <t>महाराष्ट्र</t>
         </is>
       </c>
       <c r="E282" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
     </row>
     <row r="283">
@@ -18243,20 +18366,20 @@
         </is>
       </c>
       <c r="B283" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Manipur</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>तमिलनाडु</t>
+          <t>मणिपुर</t>
         </is>
       </c>
       <c r="E283" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
     </row>
     <row r="284">
@@ -18266,20 +18389,20 @@
         </is>
       </c>
       <c r="B284" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Telangana</t>
+          <t>Meghalaya</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>तेलंगाना</t>
+          <t>मेघालय</t>
         </is>
       </c>
       <c r="E284" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
     </row>
     <row r="285">
@@ -18289,20 +18412,20 @@
         </is>
       </c>
       <c r="B285" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>Tripura</t>
+          <t>Mizoram</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>त्रिपुरा</t>
+          <t>मिज़ोरम</t>
         </is>
       </c>
       <c r="E285" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="286">
@@ -18312,20 +18435,20 @@
         </is>
       </c>
       <c r="B286" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Uttar Pradesh</t>
+          <t>Nagaland</t>
         </is>
       </c>
       <c r="D286" t="inlineStr">
         <is>
-          <t>उत्तर प्रदेश</t>
+          <t>नागालैंड</t>
         </is>
       </c>
       <c r="E286" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="287">
@@ -18335,20 +18458,20 @@
         </is>
       </c>
       <c r="B287" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>West Bengal</t>
+          <t>Odisha</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>पश्चिम बंगाल</t>
+          <t>ओडिशा</t>
         </is>
       </c>
       <c r="E287" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
     </row>
     <row r="288">
@@ -18358,20 +18481,20 @@
         </is>
       </c>
       <c r="B288" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Andaman and Nicobar Islands</t>
+          <t>Punjab</t>
         </is>
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>अंडमान और निकोबार द्वीप समूह</t>
+          <t>पंजाब</t>
         </is>
       </c>
       <c r="E288" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
     </row>
     <row r="289">
@@ -18381,20 +18504,20 @@
         </is>
       </c>
       <c r="B289" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Chandigarh</t>
+          <t>Rajasthan</t>
         </is>
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>चंडीगढ़</t>
+          <t>राजस्थान</t>
         </is>
       </c>
       <c r="E289" t="n">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="290">
@@ -18404,20 +18527,20 @@
         </is>
       </c>
       <c r="B290" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Dadra and Nagar Haveli and Daman and Diu</t>
+          <t>Sikkim</t>
         </is>
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>दादरा और नगर हवेली तथा दमन और दीव</t>
+          <t>सिक्किम</t>
         </is>
       </c>
       <c r="E290" t="n">
-        <v>31</v>
+        <v>22</v>
       </c>
     </row>
     <row r="291">
@@ -18427,20 +18550,20 @@
         </is>
       </c>
       <c r="B291" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Delhi</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>दिल्ली</t>
+          <t>तमिलनाडु</t>
         </is>
       </c>
       <c r="E291" t="n">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="292">
@@ -18450,20 +18573,20 @@
         </is>
       </c>
       <c r="B292" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Jammu and Kashmir</t>
+          <t>Telangana</t>
         </is>
       </c>
       <c r="D292" t="inlineStr">
         <is>
-          <t>जम्मू और कश्मीर</t>
+          <t>तेलंगाना</t>
         </is>
       </c>
       <c r="E292" t="n">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="293">
@@ -18473,20 +18596,20 @@
         </is>
       </c>
       <c r="B293" t="n">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Ladakh</t>
+          <t>Tripura</t>
         </is>
       </c>
       <c r="D293" t="inlineStr">
         <is>
-          <t>लद्दाख</t>
+          <t>त्रिपुरा</t>
         </is>
       </c>
       <c r="E293" t="n">
-        <v>34</v>
+        <v>25</v>
       </c>
     </row>
     <row r="294">
@@ -18496,20 +18619,20 @@
         </is>
       </c>
       <c r="B294" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Lakshadweep</t>
+          <t>Uttar Pradesh</t>
         </is>
       </c>
       <c r="D294" t="inlineStr">
         <is>
-          <t>लक्षद्वीप</t>
+          <t>उत्तर प्रदेश</t>
         </is>
       </c>
       <c r="E294" t="n">
-        <v>35</v>
+        <v>26</v>
       </c>
     </row>
     <row r="295">
@@ -18519,434 +18642,434 @@
         </is>
       </c>
       <c r="B295" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Puducherry</t>
+          <t>West Bengal</t>
         </is>
       </c>
       <c r="D295" t="inlineStr">
         <is>
-          <t>पुदुच्चेरी</t>
+          <t>पश्चिम बंगाल</t>
         </is>
       </c>
       <c r="E295" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>task3</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B296" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Yes, regularly in my main Yatra work</t>
+          <t>Andaman and Nicobar Islands</t>
         </is>
       </c>
       <c r="D296" t="inlineStr">
         <is>
-          <t>हाँ, अपने मुख्य यात्रा-काम में नियमित</t>
+          <t>अंडमान और निकोबार द्वीप समूह</t>
         </is>
       </c>
       <c r="E296" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>task3</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B297" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Not in my main work, but done before elsewhere</t>
+          <t>Chandigarh</t>
         </is>
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>मुख्य काम में नहीं, पर पहले कहीं और किया है</t>
+          <t>चंडीगढ़</t>
         </is>
       </c>
       <c r="E297" t="n">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>task3</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B298" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Never done</t>
+          <t>Dadra and Nagar Haveli and Daman and Diu</t>
         </is>
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>कभी नहीं किया</t>
+          <t>दादरा और नगर हवेली तथा दमन और दीव</t>
         </is>
       </c>
       <c r="E298" t="n">
-        <v>3</v>
+        <v>31</v>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>toilet</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B299" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>No toilet / open defecation</t>
+          <t>Delhi</t>
         </is>
       </c>
       <c r="D299" t="inlineStr">
         <is>
-          <t>शौचालय नहीं / खुले में</t>
+          <t>दिल्ली</t>
         </is>
       </c>
       <c r="E299" t="n">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>toilet</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B300" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Pit latrine without slab or open pit</t>
+          <t>Jammu and Kashmir</t>
         </is>
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>बिना ढँके गड्ढे वाला शौचालय</t>
+          <t>जम्मू और कश्मीर</t>
         </is>
       </c>
       <c r="E300" t="n">
-        <v>2</v>
+        <v>33</v>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>toilet</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B301" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Improved toilet, but shared with other households</t>
+          <t>Ladakh</t>
         </is>
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>अच्छा शौचालय, पर दूसरे घरों के साथ साझा</t>
+          <t>लद्दाख</t>
         </is>
       </c>
       <c r="E301" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>toilet</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B302" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Improved toilet, used only by this household</t>
+          <t>Lakshadweep</t>
         </is>
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>अच्छा शौचालय, सिर्फ़ इसी घर के लिए</t>
+          <t>लक्षद्वीप</t>
         </is>
       </c>
       <c r="E302" t="n">
-        <v>4</v>
+        <v>35</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B303" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Mud, thatch, bamboo or other natural material</t>
+          <t>Puducherry</t>
         </is>
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>मिट्टी, फूस, बाँस या ऐसी ही कोई चीज़</t>
+          <t>पुदुच्चेरी</t>
         </is>
       </c>
       <c r="E303" t="n">
-        <v>1</v>
+        <v>36</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>task3</t>
         </is>
       </c>
       <c r="B304" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>Unburnt brick, wood or tin</t>
+          <t>Yes, regularly in my main Yatra work</t>
         </is>
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>कच्ची ईंट, लकड़ी या टीन</t>
+          <t>हाँ, अपने मुख्य यात्रा-काम में नियमित</t>
         </is>
       </c>
       <c r="E304" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>task3</t>
         </is>
       </c>
       <c r="B305" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Burnt brick, cement, concrete or stone</t>
+          <t>Not in my main work, but done before elsewhere</t>
         </is>
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>पक्की ईंट, सीमेंट, कंक्रीट या पत्थर</t>
+          <t>मुख्य काम में नहीं, पर पहले कहीं और किया है</t>
         </is>
       </c>
       <c r="E305" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>task3</t>
         </is>
       </c>
       <c r="B306" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Piped into the house or yard</t>
+          <t>Never done</t>
         </is>
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>घर या आँगन में नल</t>
+          <t>कभी नहीं किया</t>
         </is>
       </c>
       <c r="E306" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="B307" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Public tap or standpipe</t>
+          <t>No toilet / open defecation</t>
         </is>
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>सार्वजनिक नल या स्टैंडपोस्ट</t>
+          <t>शौचालय नहीं / खुले में</t>
         </is>
       </c>
       <c r="E307" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="B308" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Handpump, tubewell or borewell</t>
+          <t>Pit latrine without slab or open pit</t>
         </is>
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>हैंडपंप, ट्यूबवेल या बोरवेल</t>
+          <t>बिना ढँके गड्ढे वाला शौचालय</t>
         </is>
       </c>
       <c r="E308" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="B309" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Protected well or protected spring</t>
+          <t>Improved toilet, but shared with other households</t>
         </is>
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>ढका हुआ कुआँ या ढका हुआ सोता</t>
+          <t>अच्छा शौचालय, पर दूसरे घरों के साथ साझा</t>
         </is>
       </c>
       <c r="E309" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>toilet</t>
         </is>
       </c>
       <c r="B310" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Rainwater collection</t>
+          <t>Improved toilet, used only by this household</t>
         </is>
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>बारिश का पानी जमा करके</t>
+          <t>अच्छा शौचालय, सिर्फ़ इसी घर के लिए</t>
         </is>
       </c>
       <c r="E310" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="B311" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>Bottled, packaged or community RO</t>
+          <t>Mud, thatch, bamboo or other natural material</t>
         </is>
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>बोतलबंद, पैकेट या सामुदायिक RO</t>
+          <t>मिट्टी, फूस, बाँस या ऐसी ही कोई चीज़</t>
         </is>
       </c>
       <c r="E311" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="B312" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Unprotected well or unprotected spring</t>
+          <t>Unburnt brick, wood or tin</t>
         </is>
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>खुला कुआँ या खुला सोता</t>
+          <t>कच्ची ईंट, लकड़ी या टीन</t>
         </is>
       </c>
       <c r="E312" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>water</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="B313" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>River, stream, pond or canal</t>
+          <t>Burnt brick, cement, concrete or stone</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>नदी, गाड़, तालाब या नहर</t>
+          <t>पक्की ईंट, सीमेंट, कंक्रीट या पत्थर</t>
         </is>
       </c>
       <c r="E313" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="314">
@@ -18956,318 +19079,502 @@
         </is>
       </c>
       <c r="B314" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Tanker truck or cart with drum</t>
+          <t>Piped into the house or yard</t>
         </is>
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>टैंकर या ड्रम वाली गाड़ी</t>
+          <t>घर या आँगन में नल</t>
         </is>
       </c>
       <c r="E314" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>wgdiff</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B315" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>No difficulty</t>
+          <t>Public tap or standpipe</t>
         </is>
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>कोई दिक़्क़त नहीं</t>
+          <t>सार्वजनिक नल या स्टैंडपोस्ट</t>
         </is>
       </c>
       <c r="E315" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>wgdiff</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B316" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Some difficulty</t>
+          <t>Handpump, tubewell or borewell</t>
         </is>
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>थोड़ी दिक़्क़त</t>
+          <t>हैंडपंप, ट्यूबवेल या बोरवेल</t>
         </is>
       </c>
       <c r="E316" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>wgdiff</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B317" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>A lot of difficulty</t>
+          <t>Protected well or protected spring</t>
         </is>
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>बहुत दिक़्क़त</t>
+          <t>ढका हुआ कुआँ या ढका हुआ सोता</t>
         </is>
       </c>
       <c r="E317" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>wgdiff</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B318" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Cannot do it at all</t>
+          <t>Rainwater collection</t>
         </is>
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>बिलकुल नहीं कर पाते</t>
+          <t>बारिश का पानी जमा करके</t>
         </is>
       </c>
       <c r="E318" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>workins</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B319" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Yes, through work</t>
+          <t>Bottled, packaged or community RO</t>
         </is>
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>हाँ, काम की तरफ़ से</t>
+          <t>बोतलबंद, पैकेट या सामुदायिक RO</t>
         </is>
       </c>
       <c r="E319" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>workins</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B320" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Only private or other insurance</t>
+          <t>Unprotected well or unprotected spring</t>
         </is>
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>सिर्फ़ अपना या कोई और बीमा</t>
+          <t>खुला कुआँ या खुला सोता</t>
         </is>
       </c>
       <c r="E320" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>workins</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B321" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>River, stream, pond or canal</t>
         </is>
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>कोई नहीं</t>
+          <t>नदी, गाड़, तालाब या नहर</t>
         </is>
       </c>
       <c r="E321" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>workins</t>
+          <t>water</t>
         </is>
       </c>
       <c r="B322" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Don't know</t>
+          <t>Tanker truck or cart with drum</t>
         </is>
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>पता नहीं</t>
+          <t>टैंकर या ड्रम वाली गाड़ी</t>
         </is>
       </c>
       <c r="E322" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>yn</t>
+          <t>wgdiff</t>
         </is>
       </c>
       <c r="B323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No difficulty</t>
         </is>
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>नहीं</t>
+          <t>कोई दिक़्क़त नहीं</t>
         </is>
       </c>
       <c r="E323" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>yn</t>
+          <t>wgdiff</t>
         </is>
       </c>
       <c r="B324" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Some difficulty</t>
         </is>
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>हाँ</t>
+          <t>थोड़ी दिक़्क़त</t>
         </is>
       </c>
       <c r="E324" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>yndk</t>
+          <t>wgdiff</t>
         </is>
       </c>
       <c r="B325" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>A lot of difficulty</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>नहीं</t>
+          <t>बहुत दिक़्क़त</t>
         </is>
       </c>
       <c r="E325" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>yndk</t>
+          <t>wgdiff</t>
         </is>
       </c>
       <c r="B326" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Cannot do it at all</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>हाँ</t>
+          <t>बिलकुल नहीं कर पाते</t>
         </is>
       </c>
       <c r="E326" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
+          <t>workins</t>
+        </is>
+      </c>
+      <c r="B327" t="n">
+        <v>1</v>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Yes, through work</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>हाँ, काम की तरफ़ से</t>
+        </is>
+      </c>
+      <c r="E327" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>workins</t>
+        </is>
+      </c>
+      <c r="B328" t="n">
+        <v>2</v>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Only private or other insurance</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>सिर्फ़ अपना या कोई और बीमा</t>
+        </is>
+      </c>
+      <c r="E328" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>workins</t>
+        </is>
+      </c>
+      <c r="B329" t="n">
+        <v>3</v>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>कोई नहीं</t>
+        </is>
+      </c>
+      <c r="E329" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>workins</t>
+        </is>
+      </c>
+      <c r="B330" t="n">
+        <v>4</v>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Don't know</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>पता नहीं</t>
+        </is>
+      </c>
+      <c r="E330" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>yn</t>
+        </is>
+      </c>
+      <c r="B331" t="n">
+        <v>0</v>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>नहीं</t>
+        </is>
+      </c>
+      <c r="E331" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>yn</t>
+        </is>
+      </c>
+      <c r="B332" t="n">
+        <v>1</v>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="E332" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
           <t>yndk</t>
         </is>
       </c>
-      <c r="B327" t="n">
+      <c r="B333" t="n">
+        <v>0</v>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>नहीं</t>
+        </is>
+      </c>
+      <c r="E333" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>yndk</t>
+        </is>
+      </c>
+      <c r="B334" t="n">
+        <v>1</v>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="E334" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>yndk</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
         <v>97</v>
       </c>
-      <c r="C327" t="inlineStr">
+      <c r="C335" t="inlineStr">
         <is>
           <t>Don't know</t>
         </is>
       </c>
-      <c r="D327" t="inlineStr">
+      <c r="D335" t="inlineStr">
         <is>
           <t>पता नहीं</t>
         </is>
       </c>
-      <c r="E327" t="n">
+      <c r="E335" t="n">
         <v>97</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Enumerator note: luggage hauling by porters and pony owners/workers
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kedarnath_final_kobo.xlsx
+++ b/Kedarnath_final_kobo.xlsx
@@ -2005,8 +2005,16 @@
           <t>वे कौन-कौन से काम हैं? जो-जो लागू हो, सब बताइए।</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ENUMERATOR: hauling luggage or goods on the back, shoulders or a head-load, for pilgrims or shops, is code 3 (porter). Carrying a person in a kandi is also code 3; carrying a person on a palanquin as part of a team is code 4. Hauling luggage or goods on a pony or mule is code 1 if the respondent works the animal for someone else, and code 2 if they own it.</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>सर्वेक्षक के लिए: पीठ, कंधे या सिर पर सामान या लगेज ढोना (तीर्थयात्रियों या दुकानों के लिए) = कोड 3 (पोर्टर)। कंडी में इंसान ढोना भी कोड 3; पालकी या डंडी टीम में ढोना कोड 4। पोनी या खच्चर पर सामान ढोना: अगर किसी और का जानवर चलाते हैं तो कोड 1, अगर जानवर खुद का है तो कोड 2।</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
           <t>yes</t>

</xml_diff>

<commit_message>
Common-land items: season recall, Yatra region, and the respondent or anyone staying with them
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Kedarnath_final_kobo.xlsx
+++ b/Kedarnath_final_kobo.xlsx
@@ -11562,12 +11562,12 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>In the last 12 months, did anyone in your household collect firewood or dead wood from common land or forest near here?</t>
+          <t>In this Yatra season or last Yatra season, did you or anyone staying with you here collect firewood or dead wood from common land or forest in the Yatra region or workplace region?</t>
         </is>
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने आस-पास की साझा ज़मीन या जंगल से लकड़ी या सूखी टहनियाँ इकट्ठी कीं?</t>
+          <t>इस यात्रा सीज़न या पिछले यात्रा सीज़न में, क्या आपने या आपके साथ यहाँ रहने वाले किसी ने यात्रा क्षेत्र या काम की जगह की साझा ज़मीन या जंगल से लकड़ी या सूखी टहनियाँ इकट्ठी कीं?</t>
         </is>
       </c>
       <c r="E280" t="inlineStr"/>
@@ -11599,12 +11599,12 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>In the last 12 months, did anyone in your household cut grass or fodder from common land near here?</t>
+          <t>In this Yatra season or last Yatra season, did you or anyone staying with you here cut grass or fodder from common land in the Yatra region or workplace region?</t>
         </is>
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने साझा ज़मीन से घास या चारा काटा?</t>
+          <t>इस यात्रा सीज़न या पिछले यात्रा सीज़न में, क्या आपने या आपके साथ यहाँ रहने वाले किसी ने यात्रा क्षेत्र या काम की जगह की साझा ज़मीन से घास या चारा काटा?</t>
         </is>
       </c>
       <c r="E281" t="inlineStr"/>
@@ -11636,12 +11636,12 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>In the last 12 months, did anyone in your household collect herbs, mushrooms or wild fruit from the forest?</t>
+          <t>In this Yatra season or last Yatra season, did you or anyone staying with you here collect herbs, mushrooms or wild fruit from the forest in the Yatra region or workplace region?</t>
         </is>
       </c>
       <c r="D282" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी ने जंगल से जड़ी-बूटी, मशरूम या जंगली फल इकट्ठे किए?</t>
+          <t>इस यात्रा सीज़न या पिछले यात्रा सीज़न में, क्या आपने या आपके साथ यहाँ रहने वाले किसी ने यात्रा क्षेत्र या काम की जगह के जंगल से जड़ी-बूटी, मशरूम या जंगली फल इकट्ठे किए?</t>
         </is>
       </c>
       <c r="E282" t="inlineStr"/>
@@ -11673,12 +11673,12 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>In the last 12 months, did any animal of your household graze on common pasture?</t>
+          <t>In this Yatra season or last Yatra season, did any animal of yours or of anyone staying with you here graze on common pasture in the Yatra region or workplace region?</t>
         </is>
       </c>
       <c r="D283" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर का कोई जानवर साझा चरागाह में चरा?</t>
+          <t>इस यात्रा सीज़न या पिछले यात्रा सीज़न में, क्या आपका या आपके साथ यहाँ रहने वाले किसी का कोई जानवर यात्रा क्षेत्र या काम की जगह की साझा चरागाह में चरा?</t>
         </is>
       </c>
       <c r="E283" t="inlineStr"/>
@@ -11710,12 +11710,12 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>In the last 12 months, has anyone in your household been stopped from using a common forest, pasture or path, or been asked to pay to use it?</t>
+          <t>In this Yatra season or last Yatra season, has anyone you or someone staying with you here been stopped from using a common forest, pasture or path, or been asked to pay to use it, in the Yatra region or workplace region?</t>
         </is>
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या आपके घर के किसी को साझा जंगल, चरागाह या रास्ते के इस्तेमाल से रोका गया, या इसके लिए पैसे देने को कहा गया?</t>
+          <t>इस यात्रा सीज़न या पिछले यात्रा सीज़न में, क्या आपको या आपके साथ यहाँ रहने वाले किसी को यात्रा क्षेत्र या काम की जगह में साझा जंगल, चरागाह या रास्ते के इस्तेमाल से रोका गया, या इसके लिए पैसे देने को कहा गया?</t>
         </is>
       </c>
       <c r="E284" t="inlineStr"/>
@@ -11747,12 +11747,12 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>In the last 12 months, has a common place you used to collect from or graze on been closed because of building, road or ropeway work?</t>
+          <t>In this Yatra season or last Yatra season, has a common place you used to collect from or graze on been closed, because of a landslide, flood, road or bridge damage, or construction work, in the Yatra region or workplace region?</t>
         </is>
       </c>
       <c r="D285" t="inlineStr">
         <is>
-          <t>पिछले 12 महीनों में, क्या कोई साझा जगह, जहाँ आप पहले लकड़ी, घास या चारा लेते थे, निर्माण, सड़क या रोपवे के काम की वजह से बंद हो गई?</t>
+          <t>इस यात्रा सीज़न या पिछले यात्रा सीज़न में, क्या कोई साझा जगह, जहाँ आप पहले लकड़ी, घास या चारा लेते थे, भूस्खलन, बाढ़, सड़क या पुल टूटने, या निर्माण कार्य की वजह से बंद हो गई?</t>
         </is>
       </c>
       <c r="E285" t="inlineStr"/>
@@ -11821,12 +11821,12 @@
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>In this area, who decides who may use the common land and forest? Ask and code what they name; do not read the list.</t>
+          <t>In the Yatra region or workplace region, who decides who may use the common land and forest? Ask and code what they name; do not read the list.</t>
         </is>
       </c>
       <c r="D287" t="inlineStr">
         <is>
-          <t>इस इलाके की साझा ज़मीन और जंगल का फ़ैसला कौन करता है, कि कौन उसका इस्तेमाल कर सकता है? जो नाम लें वही लिख लें; सूची न पढ़ें।</t>
+          <t>यात्रा क्षेत्र या काम की जगह की साझा ज़मीन और जंगल का फ़ैसला कौन करता है, कि कौन उसका इस्तेमाल कर सकता है? जो नाम लें वही लिख लें; सूची न पढ़ें।</t>
         </is>
       </c>
       <c r="E287" t="inlineStr"/>

</xml_diff>